<commit_message>
Estadisticos Segundo Parcial 20241 Martes
</commit_message>
<xml_diff>
--- a/Totales Generales20241.xlsx
+++ b/Totales Generales20241.xlsx
@@ -644,22 +644,22 @@
         <v>9</v>
       </c>
       <c r="K2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M2">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P2" s="1">
-        <v>46.8</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -691,25 +691,25 @@
         <v>2</v>
       </c>
       <c r="J3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L3">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M3">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="N3">
-        <v>101</v>
+        <v>126</v>
       </c>
       <c r="O3">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="P3" s="1">
-        <v>45.1</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -747,10 +747,10 @@
         <v>6</v>
       </c>
       <c r="L4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M4">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N4">
         <v>148</v>
@@ -791,25 +791,25 @@
         <v>14</v>
       </c>
       <c r="J5">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K5">
         <v>31</v>
       </c>
       <c r="L5">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M5">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="N5">
-        <v>374</v>
+        <v>400</v>
       </c>
       <c r="O5">
-        <v>255</v>
+        <v>229</v>
       </c>
       <c r="P5" s="1">
-        <v>40.5</v>
+        <v>36.4</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -838,28 +838,28 @@
         <v>4</v>
       </c>
       <c r="I6">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K6">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M6">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N6">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O6">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P6" s="1">
-        <v>75.2</v>
+        <v>74.5</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -988,28 +988,28 @@
         <v>7</v>
       </c>
       <c r="I9">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J9">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K9">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L9">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M9">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N9">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="O9">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="P9" s="1">
-        <v>60.4</v>
+        <v>60.1</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -1035,28 +1035,28 @@
         <v>19</v>
       </c>
       <c r="I10">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J10">
         <v>38</v>
       </c>
       <c r="K10">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L10">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M10">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="N10">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="O10">
-        <v>473</v>
+        <v>446</v>
       </c>
       <c r="P10" s="1">
-        <v>47.8</v>
+        <v>45.1</v>
       </c>
     </row>
   </sheetData>
@@ -1139,25 +1139,25 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -1189,37 +1189,37 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>184</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L3">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="M3">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="N3">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="O3">
-        <v>184</v>
+        <v>127</v>
       </c>
       <c r="P3" s="1">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -1242,25 +1242,25 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>151</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L4">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1289,37 +1289,37 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>419</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>59</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <v>151</v>
+        <v>9</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>154</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>244</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="O5">
-        <v>629</v>
+        <v>572</v>
       </c>
       <c r="P5" s="1">
-        <v>100</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1339,28 +1339,28 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>148</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1389,37 +1389,37 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="M7">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O7">
-        <v>97</v>
+        <v>57</v>
       </c>
       <c r="P7" s="1">
-        <v>100</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -1442,34 +1442,34 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H8">
-        <v>94</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L8">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="M8">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="O8">
-        <v>115</v>
+        <v>65</v>
       </c>
       <c r="P8" s="1">
-        <v>100</v>
+        <v>56.5</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -1489,37 +1489,37 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>244</v>
+        <v>6</v>
       </c>
       <c r="G9">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="H9">
-        <v>95</v>
+        <v>18</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="K9">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="L9">
-        <v>1</v>
+        <v>78</v>
       </c>
       <c r="M9">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="N9">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="O9">
-        <v>361</v>
+        <v>271</v>
       </c>
       <c r="P9" s="1">
-        <v>100</v>
+        <v>75.09999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -1536,37 +1536,37 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>663</v>
+        <v>6</v>
       </c>
       <c r="G10">
-        <v>79</v>
+        <v>12</v>
       </c>
       <c r="H10">
-        <v>246</v>
+        <v>27</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>134</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>232</v>
       </c>
       <c r="M10">
-        <v>0</v>
+        <v>332</v>
       </c>
       <c r="N10">
-        <v>0</v>
+        <v>147</v>
       </c>
       <c r="O10">
-        <v>990</v>
+        <v>843</v>
       </c>
       <c r="P10" s="1">
-        <v>100</v>
+        <v>85.2</v>
       </c>
     </row>
   </sheetData>
@@ -1649,37 +1649,37 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2">
         <v>6</v>
       </c>
       <c r="I2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J2">
         <v>9</v>
       </c>
       <c r="K2">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="L2">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="M2">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="N2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P2" s="1">
-        <v>46.8</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -1702,25 +1702,25 @@
         <v>0</v>
       </c>
       <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="J3">
         <v>2</v>
       </c>
-      <c r="H3">
-        <v>3</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>4</v>
-      </c>
       <c r="K3">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="L3">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="M3">
-        <v>101</v>
+        <v>149</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1752,34 +1752,34 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I4">
         <v>3</v>
       </c>
       <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
         <v>4</v>
       </c>
-      <c r="K4">
-        <v>6</v>
-      </c>
       <c r="L4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M4">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="N4">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="O4">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="P4" s="1">
-        <v>29.5</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -1799,37 +1799,37 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5">
         <v>6</v>
       </c>
-      <c r="H5">
-        <v>12</v>
-      </c>
       <c r="I5">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J5">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K5">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="L5">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="M5">
-        <v>175</v>
+        <v>236</v>
       </c>
       <c r="N5">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="O5">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="P5" s="1">
-        <v>56.6</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1852,34 +1852,34 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I6">
+        <v>14</v>
+      </c>
+      <c r="J6">
+        <v>16</v>
+      </c>
+      <c r="K6">
         <v>18</v>
       </c>
-      <c r="J6">
+      <c r="L6">
         <v>13</v>
       </c>
-      <c r="K6">
-        <v>17</v>
-      </c>
-      <c r="L6">
-        <v>20</v>
-      </c>
       <c r="M6">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="N6">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="O6">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="P6" s="1">
-        <v>75.2</v>
+        <v>65.8</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -1899,28 +1899,28 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I7">
         <v>5</v>
       </c>
       <c r="J7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K7">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="L7">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="M7">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -1955,31 +1955,31 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <v>4</v>
       </c>
       <c r="K8">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="L8">
         <v>9</v>
       </c>
       <c r="M8">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N8">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="O8">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="P8" s="1">
-        <v>45.2</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -1999,37 +1999,37 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G9">
+        <v>6</v>
+      </c>
+      <c r="H9">
         <v>10</v>
       </c>
-      <c r="H9">
-        <v>8</v>
-      </c>
       <c r="I9">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="J9">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K9">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="L9">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="M9">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="N9">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="O9">
-        <v>260</v>
+        <v>230</v>
       </c>
       <c r="P9" s="1">
-        <v>72</v>
+        <v>63.7</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -2049,34 +2049,34 @@
         <v>3</v>
       </c>
       <c r="G10">
+        <v>9</v>
+      </c>
+      <c r="H10">
         <v>16</v>
       </c>
-      <c r="H10">
-        <v>20</v>
-      </c>
       <c r="I10">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="J10">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="K10">
-        <v>97</v>
+        <v>58</v>
       </c>
       <c r="L10">
-        <v>128</v>
+        <v>98</v>
       </c>
       <c r="M10">
-        <v>270</v>
+        <v>334</v>
       </c>
       <c r="N10">
-        <v>374</v>
+        <v>408</v>
       </c>
       <c r="O10">
-        <v>616</v>
+        <v>582</v>
       </c>
       <c r="P10" s="1">
-        <v>62.2</v>
+        <v>58.8</v>
       </c>
     </row>
   </sheetData>
@@ -2156,34 +2156,34 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="M2">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N2">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="O2" s="1">
-        <v>40</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -2200,28 +2200,28 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3">
         <v>2</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="J3">
         <v>3</v>
       </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>6</v>
-      </c>
       <c r="K3">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L3">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M3">
         <v>0</v>
@@ -2253,31 +2253,31 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
         <v>6</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>8</v>
       </c>
-      <c r="L4">
-        <v>3</v>
-      </c>
       <c r="M4">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O4" s="1">
-        <v>37.5</v>
+        <v>35.4</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -2306,25 +2306,25 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
         <v>2</v>
       </c>
-      <c r="L5">
-        <v>4</v>
-      </c>
       <c r="M5">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="N5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O5" s="1">
-        <v>27.8</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -2347,31 +2347,31 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J6">
         <v>2</v>
       </c>
       <c r="K6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N6">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O6" s="1">
-        <v>37.8</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -2397,19 +2397,19 @@
         <v>2</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7">
         <v>4</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M7">
         <v>22</v>
@@ -2438,25 +2438,25 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L8">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="M8">
         <v>0</v>
@@ -2497,13 +2497,13 @@
         <v>0</v>
       </c>
       <c r="J9">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K9">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L9">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="M9">
         <v>0</v>
@@ -2532,25 +2532,25 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="M10">
         <v>0</v>
@@ -2579,7 +2579,7 @@
         <v>0</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -2591,13 +2591,13 @@
         <v>0</v>
       </c>
       <c r="J11">
+        <v>2</v>
+      </c>
+      <c r="K11">
         <v>3</v>
       </c>
-      <c r="K11">
-        <v>2</v>
-      </c>
       <c r="L11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M11">
         <v>0</v>
@@ -2632,7 +2632,7 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12">
         <v>1</v>
@@ -2641,10 +2641,10 @@
         <v>5</v>
       </c>
       <c r="K12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L12">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M12">
         <v>0</v>
@@ -2676,22 +2676,22 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
         <v>2</v>
       </c>
-      <c r="J13">
-        <v>1</v>
-      </c>
       <c r="K13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L13">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="M13">
         <v>0</v>
@@ -2720,22 +2720,22 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L14">
         <v>3</v>
@@ -2779,22 +2779,22 @@
         <v>0</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L15">
+        <v>5</v>
+      </c>
+      <c r="M15">
+        <v>34</v>
+      </c>
+      <c r="N15">
         <v>7</v>
       </c>
-      <c r="M15">
-        <v>33</v>
-      </c>
-      <c r="N15">
-        <v>8</v>
-      </c>
       <c r="O15" s="1">
-        <v>19.5</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -2820,16 +2820,16 @@
         <v>0</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L16">
         <v>9</v>
@@ -2876,10 +2876,10 @@
         <v>0</v>
       </c>
       <c r="K17">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L17">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="M17">
         <v>27</v>
@@ -2911,31 +2911,31 @@
         <v>0</v>
       </c>
       <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
         <v>2</v>
       </c>
-      <c r="H18">
-        <v>2</v>
-      </c>
-      <c r="I18">
-        <v>2</v>
-      </c>
-      <c r="J18">
+      <c r="K18">
         <v>3</v>
       </c>
-      <c r="K18">
-        <v>2</v>
-      </c>
       <c r="L18">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M18">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="N18">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="O18" s="1">
-        <v>41.9</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -3002,34 +3002,34 @@
         <v>0</v>
       </c>
       <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>6</v>
+      </c>
+      <c r="I20">
+        <v>4</v>
+      </c>
+      <c r="J20">
+        <v>6</v>
+      </c>
+      <c r="K20">
         <v>2</v>
       </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="H20">
-        <v>7</v>
-      </c>
-      <c r="I20">
-        <v>6</v>
-      </c>
-      <c r="J20">
-        <v>4</v>
-      </c>
-      <c r="K20">
-        <v>8</v>
-      </c>
       <c r="L20">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M20">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="N20">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="O20" s="1">
-        <v>90</v>
+        <v>72.5</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -3049,25 +3049,25 @@
         <v>0</v>
       </c>
       <c r="F21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J21">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K21">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L21">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M21">
         <v>7</v>
@@ -3102,28 +3102,28 @@
         <v>3</v>
       </c>
       <c r="H22">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L22">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M22">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="N22">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="O22" s="1">
-        <v>66.7</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -3143,22 +3143,22 @@
         <v>0</v>
       </c>
       <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
         <v>2</v>
-      </c>
-      <c r="G23">
-        <v>0</v>
       </c>
       <c r="H23">
         <v>3</v>
       </c>
       <c r="I23">
+        <v>3</v>
+      </c>
+      <c r="J23">
+        <v>3</v>
+      </c>
+      <c r="K23">
         <v>4</v>
-      </c>
-      <c r="J23">
-        <v>1</v>
-      </c>
-      <c r="K23">
-        <v>5</v>
       </c>
       <c r="L23">
         <v>3</v>
@@ -3196,19 +3196,19 @@
         <v>0</v>
       </c>
       <c r="H24">
+        <v>1</v>
+      </c>
+      <c r="I24">
         <v>2</v>
       </c>
-      <c r="I24">
-        <v>1</v>
-      </c>
       <c r="J24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M24">
         <v>10</v>
@@ -3234,28 +3234,28 @@
         <v>0</v>
       </c>
       <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
         <v>2</v>
       </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-      <c r="G25">
+      <c r="H25">
         <v>4</v>
       </c>
-      <c r="H25">
-        <v>1</v>
-      </c>
       <c r="I25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M25">
         <v>1</v>
@@ -3290,19 +3290,19 @@
         <v>0</v>
       </c>
       <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>1</v>
+      </c>
+      <c r="J26">
         <v>2</v>
       </c>
-      <c r="I26">
-        <v>2</v>
-      </c>
-      <c r="J26">
-        <v>7</v>
-      </c>
       <c r="K26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L26">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="M26">
         <v>0</v>
@@ -3340,16 +3340,16 @@
         <v>1</v>
       </c>
       <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
         <v>2</v>
       </c>
-      <c r="J27">
-        <v>3</v>
-      </c>
       <c r="K27">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L27">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M27">
         <v>0</v>
@@ -3384,19 +3384,19 @@
         <v>0</v>
       </c>
       <c r="H28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L28">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M28">
         <v>0</v>
@@ -3440,10 +3440,10 @@
         <v>0</v>
       </c>
       <c r="K29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M29">
         <v>0</v>
@@ -3475,31 +3475,31 @@
         <v>0</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L30">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M30">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N30">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="O30" s="1">
-        <v>61.9</v>
+        <v>52.4</v>
       </c>
     </row>
     <row r="31" spans="1:15">
@@ -3522,31 +3522,31 @@
         <v>0</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
         <v>2</v>
       </c>
-      <c r="J31">
+      <c r="K31">
         <v>4</v>
-      </c>
-      <c r="K31">
-        <v>2</v>
       </c>
       <c r="L31">
         <v>6</v>
       </c>
       <c r="M31">
+        <v>15</v>
+      </c>
+      <c r="N31">
         <v>13</v>
       </c>
-      <c r="N31">
-        <v>15</v>
-      </c>
       <c r="O31" s="1">
-        <v>53.6</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="32" spans="1:15">
@@ -3572,28 +3572,28 @@
         <v>0</v>
       </c>
       <c r="H32">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I32">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J32">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M32">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N32">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O32" s="1">
-        <v>44.4</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="33" spans="1:15">
@@ -3625,22 +3625,22 @@
         <v>0</v>
       </c>
       <c r="J33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33">
         <v>1</v>
       </c>
       <c r="L33">
+        <v>3</v>
+      </c>
+      <c r="M33">
+        <v>19</v>
+      </c>
+      <c r="N33">
         <v>4</v>
       </c>
-      <c r="M33">
-        <v>17</v>
-      </c>
-      <c r="N33">
-        <v>6</v>
-      </c>
       <c r="O33" s="1">
-        <v>26.1</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="34" spans="1:15">
@@ -3672,22 +3672,22 @@
         <v>0</v>
       </c>
       <c r="J34">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K34">
         <v>0</v>
       </c>
       <c r="L34">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M34">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="N34">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="O34" s="1">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F2" s="1">
         <v>60</v>
@@ -3752,7 +3752,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="1">
-        <v>60</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -3795,7 +3795,7 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F4" s="1">
         <v>62.5</v>
@@ -3804,7 +3804,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="1">
-        <v>62.5</v>
+        <v>64.59999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -3821,7 +3821,7 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F5" s="1">
         <v>72.2</v>
@@ -3830,7 +3830,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="1">
-        <v>72.2</v>
+        <v>77.8</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3841,22 +3841,22 @@
         <v>37</v>
       </c>
       <c r="C6">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F6" s="1">
-        <v>62.2</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
       </c>
       <c r="H6" s="1">
-        <v>62.2</v>
+        <v>64.90000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -3922,7 +3922,7 @@
         <v>18</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -3931,7 +3931,7 @@
         <v>50</v>
       </c>
       <c r="G9" s="1">
-        <v>0</v>
+        <v>77.8</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
@@ -3945,7 +3945,7 @@
         <v>28</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -3954,7 +3954,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="1">
-        <v>0</v>
+        <v>89.3</v>
       </c>
       <c r="G10" s="1">
         <v>0</v>
@@ -3974,7 +3974,7 @@
         <v>28</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -3983,7 +3983,7 @@
         <v>80</v>
       </c>
       <c r="G11" s="1">
-        <v>0</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="H11" s="1">
         <v>0</v>
@@ -4081,7 +4081,7 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F15" s="1">
         <v>80.5</v>
@@ -4090,7 +4090,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="1">
-        <v>80.5</v>
+        <v>82.90000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -4159,7 +4159,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F18" s="1">
         <v>58.1</v>
@@ -4168,7 +4168,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="1">
-        <v>58.1</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -4211,7 +4211,7 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F20" s="1">
         <v>10</v>
@@ -4220,7 +4220,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="1">
-        <v>10</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -4257,22 +4257,22 @@
         <v>33</v>
       </c>
       <c r="C22">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D22">
         <v>0</v>
       </c>
       <c r="E22">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F22" s="1">
-        <v>33.3</v>
+        <v>36.4</v>
       </c>
       <c r="G22" s="1">
         <v>0</v>
       </c>
       <c r="H22" s="1">
-        <v>33.3</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -4338,7 +4338,7 @@
         <v>6</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -4347,7 +4347,7 @@
         <v>27.3</v>
       </c>
       <c r="G25" s="1">
-        <v>0</v>
+        <v>31.8</v>
       </c>
       <c r="H25" s="1">
         <v>4.5</v>
@@ -4364,7 +4364,7 @@
         <v>7</v>
       </c>
       <c r="D26">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -4373,7 +4373,7 @@
         <v>28</v>
       </c>
       <c r="G26" s="1">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="H26" s="1">
         <v>0</v>
@@ -4416,7 +4416,7 @@
         <v>15</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -4425,7 +4425,7 @@
         <v>71.40000000000001</v>
       </c>
       <c r="G28" s="1">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="H28" s="1">
         <v>0</v>
@@ -4471,7 +4471,7 @@
         <v>0</v>
       </c>
       <c r="E30">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F30" s="1">
         <v>38.1</v>
@@ -4480,7 +4480,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="1">
-        <v>38.1</v>
+        <v>47.6</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -4497,7 +4497,7 @@
         <v>0</v>
       </c>
       <c r="E31">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F31" s="1">
         <v>46.4</v>
@@ -4506,7 +4506,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="1">
-        <v>46.4</v>
+        <v>53.6</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -4520,19 +4520,19 @@
         <v>10</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E32">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F32" s="1">
         <v>55.6</v>
       </c>
       <c r="G32" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="H32" s="1">
-        <v>55.6</v>
+        <v>72.2</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -4546,19 +4546,19 @@
         <v>17</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E33">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F33" s="1">
         <v>73.90000000000001</v>
       </c>
       <c r="G33" s="1">
-        <v>0</v>
+        <v>78.3</v>
       </c>
       <c r="H33" s="1">
-        <v>73.90000000000001</v>
+        <v>82.59999999999999</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -4572,19 +4572,19 @@
         <v>15</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E34">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F34" s="1">
         <v>60</v>
       </c>
       <c r="G34" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H34" s="1">
-        <v>60</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Estadisticos Segundo Parcial 20241 Noche Miércoles
</commit_message>
<xml_diff>
--- a/Totales Generales20241.xlsx
+++ b/Totales Generales20241.xlsx
@@ -1142,34 +1142,34 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H2">
+        <v>4</v>
+      </c>
+      <c r="I2">
+        <v>11</v>
+      </c>
+      <c r="J2">
         <v>8</v>
       </c>
-      <c r="I2">
-        <v>13</v>
-      </c>
-      <c r="J2">
-        <v>23</v>
-      </c>
       <c r="K2">
-        <v>102</v>
+        <v>9</v>
       </c>
       <c r="L2">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="O2">
-        <v>235</v>
+        <v>104</v>
       </c>
       <c r="P2" s="1">
-        <v>100</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -1198,28 +1198,28 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="M3">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="N3">
-        <v>57</v>
+        <v>148</v>
       </c>
       <c r="O3">
-        <v>127</v>
+        <v>36</v>
       </c>
       <c r="P3" s="1">
-        <v>69</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -1254,13 +1254,13 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L4">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="M4">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1292,34 +1292,34 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H5">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J5">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="K5">
-        <v>115</v>
+        <v>13</v>
       </c>
       <c r="L5">
-        <v>154</v>
+        <v>51</v>
       </c>
       <c r="M5">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="N5">
-        <v>57</v>
+        <v>279</v>
       </c>
       <c r="O5">
-        <v>572</v>
+        <v>350</v>
       </c>
       <c r="P5" s="1">
-        <v>90.90000000000001</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1345,31 +1345,31 @@
         <v>2</v>
       </c>
       <c r="H6">
+        <v>14</v>
+      </c>
+      <c r="I6">
         <v>15</v>
       </c>
-      <c r="I6">
-        <v>18</v>
-      </c>
       <c r="J6">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K6">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L6">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="M6">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="O6">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="P6" s="1">
-        <v>100</v>
+        <v>87.2</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -1407,19 +1407,19 @@
         <v>1</v>
       </c>
       <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
         <v>19</v>
       </c>
-      <c r="M7">
-        <v>26</v>
-      </c>
       <c r="N7">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="O7">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="P7" s="1">
-        <v>58.8</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -1442,34 +1442,34 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L8">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="M8">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="N8">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="O8">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="P8" s="1">
-        <v>56.5</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -1492,34 +1492,34 @@
         <v>6</v>
       </c>
       <c r="G9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H9">
         <v>18</v>
       </c>
       <c r="I9">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="J9">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="K9">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="L9">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="M9">
-        <v>88</v>
+        <v>55</v>
       </c>
       <c r="N9">
-        <v>90</v>
+        <v>160</v>
       </c>
       <c r="O9">
-        <v>271</v>
+        <v>201</v>
       </c>
       <c r="P9" s="1">
-        <v>75.09999999999999</v>
+        <v>55.7</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -1539,34 +1539,34 @@
         <v>6</v>
       </c>
       <c r="G10">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H10">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="I10">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="J10">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="K10">
-        <v>134</v>
+        <v>38</v>
       </c>
       <c r="L10">
-        <v>232</v>
+        <v>98</v>
       </c>
       <c r="M10">
-        <v>332</v>
+        <v>308</v>
       </c>
       <c r="N10">
-        <v>147</v>
+        <v>439</v>
       </c>
       <c r="O10">
-        <v>843</v>
+        <v>551</v>
       </c>
       <c r="P10" s="1">
-        <v>85.2</v>
+        <v>55.7</v>
       </c>
     </row>
   </sheetData>
@@ -1649,7 +1649,7 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
         <v>2</v>
@@ -1658,28 +1658,28 @@
         <v>6</v>
       </c>
       <c r="I2">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K2">
         <v>9</v>
       </c>
       <c r="L2">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="M2">
         <v>46</v>
       </c>
       <c r="N2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P2" s="1">
-        <v>46.4</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -1699,28 +1699,28 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="M3">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1755,31 +1755,31 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M4">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N4">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="O4">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="P4" s="1">
-        <v>28.1</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -1799,37 +1799,37 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J5">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K5">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L5">
         <v>55</v>
       </c>
       <c r="M5">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="N5">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="O5">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="P5" s="1">
-        <v>56</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1861,25 +1861,25 @@
         <v>14</v>
       </c>
       <c r="J6">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K6">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L6">
         <v>13</v>
       </c>
       <c r="M6">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="N6">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="O6">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="P6" s="1">
-        <v>65.8</v>
+        <v>63.1</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -1917,10 +1917,10 @@
         <v>7</v>
       </c>
       <c r="L7">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="M7">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -1964,22 +1964,22 @@
         <v>4</v>
       </c>
       <c r="K8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L8">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M8">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="N8">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O8">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="P8" s="1">
-        <v>31.3</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -2011,25 +2011,25 @@
         <v>19</v>
       </c>
       <c r="J9">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K9">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L9">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="M9">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="N9">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="O9">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="P9" s="1">
-        <v>63.7</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -2046,37 +2046,37 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H10">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I10">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J10">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="K10">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L10">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="M10">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="N10">
-        <v>408</v>
+        <v>418</v>
       </c>
       <c r="O10">
-        <v>582</v>
+        <v>572</v>
       </c>
       <c r="P10" s="1">
-        <v>58.8</v>
+        <v>57.8</v>
       </c>
     </row>
   </sheetData>
@@ -2159,10 +2159,10 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -2171,10 +2171,10 @@
         <v>1</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M2">
         <v>21</v>
@@ -2200,25 +2200,25 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L3">
         <v>21</v>
@@ -2256,28 +2256,28 @@
         <v>1</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L4">
         <v>8</v>
       </c>
       <c r="M4">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O4" s="1">
-        <v>35.4</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -2303,28 +2303,28 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
       <c r="J5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K5">
         <v>4</v>
       </c>
       <c r="L5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M5">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O5" s="1">
-        <v>22.2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -2344,25 +2344,25 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6">
         <v>2</v>
       </c>
       <c r="K6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M6">
         <v>24</v>
@@ -2397,28 +2397,28 @@
         <v>2</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="K7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M7">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="N7">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O7" s="1">
-        <v>33.3</v>
+        <v>24.2</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -2444,10 +2444,10 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -2529,19 +2529,19 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -2635,16 +2635,16 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L12">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M12">
         <v>0</v>
@@ -2682,13 +2682,13 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13">
         <v>2</v>
       </c>
       <c r="K13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L13">
         <v>33</v>
@@ -2817,31 +2817,31 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I16">
         <v>0</v>
       </c>
       <c r="J16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L16">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M16">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="N16">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O16" s="1">
-        <v>41.2</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -3058,16 +3058,16 @@
         <v>3</v>
       </c>
       <c r="I21">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J21">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K21">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M21">
         <v>7</v>
@@ -3158,19 +3158,19 @@
         <v>3</v>
       </c>
       <c r="K23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L23">
         <v>3</v>
       </c>
       <c r="M23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N23">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O23" s="1">
-        <v>78.3</v>
+        <v>73.90000000000001</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -3208,16 +3208,16 @@
         <v>0</v>
       </c>
       <c r="L24">
+        <v>3</v>
+      </c>
+      <c r="M24">
+        <v>13</v>
+      </c>
+      <c r="N24">
         <v>6</v>
       </c>
-      <c r="M24">
-        <v>10</v>
-      </c>
-      <c r="N24">
-        <v>9</v>
-      </c>
       <c r="O24" s="1">
-        <v>47.4</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="25" spans="1:15">
@@ -3440,10 +3440,10 @@
         <v>0</v>
       </c>
       <c r="K29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L29">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M29">
         <v>0</v>
@@ -3484,10 +3484,10 @@
         <v>0</v>
       </c>
       <c r="J30">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K30">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L30">
         <v>3</v>
@@ -3537,16 +3537,16 @@
         <v>4</v>
       </c>
       <c r="L31">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M31">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="N31">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O31" s="1">
-        <v>46.4</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="32" spans="1:15">
@@ -3740,7 +3740,7 @@
         <v>24</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E2">
         <v>21</v>
@@ -3749,7 +3749,7 @@
         <v>60</v>
       </c>
       <c r="G2" s="1">
-        <v>0</v>
+        <v>62.5</v>
       </c>
       <c r="H2" s="1">
         <v>52.5</v>
@@ -3792,19 +3792,19 @@
         <v>30</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E4">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F4" s="1">
         <v>62.5</v>
       </c>
       <c r="G4" s="1">
-        <v>0</v>
+        <v>62.5</v>
       </c>
       <c r="H4" s="1">
-        <v>64.59999999999999</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -3818,19 +3818,19 @@
         <v>26</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E5">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F5" s="1">
         <v>72.2</v>
       </c>
       <c r="G5" s="1">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H5" s="1">
-        <v>77.8</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3844,7 +3844,7 @@
         <v>24</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E6">
         <v>24</v>
@@ -3853,7 +3853,7 @@
         <v>64.90000000000001</v>
       </c>
       <c r="G6" s="1">
-        <v>0</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="H6" s="1">
         <v>64.90000000000001</v>
@@ -3870,19 +3870,19 @@
         <v>22</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E7">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F7" s="1">
         <v>66.7</v>
       </c>
       <c r="G7" s="1">
-        <v>0</v>
+        <v>75.8</v>
       </c>
       <c r="H7" s="1">
-        <v>66.7</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -3896,7 +3896,7 @@
         <v>10</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -3905,7 +3905,7 @@
         <v>41.7</v>
       </c>
       <c r="G8" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
@@ -3948,7 +3948,7 @@
         <v>25</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -3957,7 +3957,7 @@
         <v>89.3</v>
       </c>
       <c r="G10" s="1">
-        <v>0</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="H10" s="1">
         <v>0</v>
@@ -4000,7 +4000,7 @@
         <v>15</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -4009,7 +4009,7 @@
         <v>62.5</v>
       </c>
       <c r="G12" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="H12" s="1">
         <v>0</v>
@@ -4026,7 +4026,7 @@
         <v>30</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -4035,7 +4035,7 @@
         <v>81.09999999999999</v>
       </c>
       <c r="G13" s="1">
-        <v>0</v>
+        <v>89.2</v>
       </c>
       <c r="H13" s="1">
         <v>0</v>
@@ -4107,7 +4107,7 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F16" s="1">
         <v>58.8</v>
@@ -4116,7 +4116,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="1">
-        <v>58.8</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -4286,19 +4286,19 @@
         <v>5</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F23" s="1">
         <v>21.7</v>
       </c>
       <c r="G23" s="1">
-        <v>0</v>
+        <v>26.1</v>
       </c>
       <c r="H23" s="1">
-        <v>21.7</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -4312,19 +4312,19 @@
         <v>10</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E24">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F24" s="1">
         <v>52.6</v>
       </c>
       <c r="G24" s="1">
-        <v>0</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="H24" s="1">
-        <v>52.6</v>
+        <v>68.40000000000001</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -4390,7 +4390,7 @@
         <v>10</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -4399,7 +4399,7 @@
         <v>52.6</v>
       </c>
       <c r="G27" s="1">
-        <v>0</v>
+        <v>57.9</v>
       </c>
       <c r="H27" s="1">
         <v>0</v>
@@ -4442,7 +4442,7 @@
         <v>5</v>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -4451,7 +4451,7 @@
         <v>50</v>
       </c>
       <c r="G29" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H29" s="1">
         <v>0</v>
@@ -4468,7 +4468,7 @@
         <v>8</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E30">
         <v>10</v>
@@ -4477,7 +4477,7 @@
         <v>38.1</v>
       </c>
       <c r="G30" s="1">
-        <v>0</v>
+        <v>47.6</v>
       </c>
       <c r="H30" s="1">
         <v>47.6</v>
@@ -4494,19 +4494,19 @@
         <v>13</v>
       </c>
       <c r="D31">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E31">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F31" s="1">
         <v>46.4</v>
       </c>
       <c r="G31" s="1">
-        <v>0</v>
+        <v>64.3</v>
       </c>
       <c r="H31" s="1">
-        <v>53.6</v>
+        <v>64.3</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -4520,7 +4520,7 @@
         <v>10</v>
       </c>
       <c r="D32">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E32">
         <v>13</v>
@@ -4529,7 +4529,7 @@
         <v>55.6</v>
       </c>
       <c r="G32" s="1">
-        <v>66.7</v>
+        <v>72.2</v>
       </c>
       <c r="H32" s="1">
         <v>72.2</v>
@@ -4546,7 +4546,7 @@
         <v>17</v>
       </c>
       <c r="D33">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E33">
         <v>19</v>
@@ -4555,7 +4555,7 @@
         <v>73.90000000000001</v>
       </c>
       <c r="G33" s="1">
-        <v>78.3</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="H33" s="1">
         <v>82.59999999999999</v>
@@ -4572,7 +4572,7 @@
         <v>15</v>
       </c>
       <c r="D34">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E34">
         <v>22</v>
@@ -4581,7 +4581,7 @@
         <v>60</v>
       </c>
       <c r="G34" s="1">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H34" s="1">
         <v>88</v>

</xml_diff>

<commit_message>
Estadisticos Segundo Parcial 20241 Miercoles Tarde
</commit_message>
<xml_diff>
--- a/Totales Generales20241.xlsx
+++ b/Totales Generales20241.xlsx
@@ -638,28 +638,28 @@
         <v>6</v>
       </c>
       <c r="I2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K2">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="L2">
         <v>23</v>
       </c>
       <c r="M2">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="N2">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="O2">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="P2" s="1">
-        <v>46.4</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -788,28 +788,28 @@
         <v>12</v>
       </c>
       <c r="I5">
+        <v>13</v>
+      </c>
+      <c r="J5">
         <v>14</v>
       </c>
-      <c r="J5">
-        <v>15</v>
-      </c>
       <c r="K5">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="L5">
         <v>55</v>
       </c>
       <c r="M5">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="N5">
-        <v>400</v>
+        <v>423</v>
       </c>
       <c r="O5">
-        <v>229</v>
+        <v>206</v>
       </c>
       <c r="P5" s="1">
-        <v>36.4</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1035,28 +1035,28 @@
         <v>19</v>
       </c>
       <c r="I10">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J10">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K10">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="L10">
         <v>100</v>
       </c>
       <c r="M10">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="N10">
-        <v>544</v>
+        <v>567</v>
       </c>
       <c r="O10">
-        <v>446</v>
+        <v>423</v>
       </c>
       <c r="P10" s="1">
-        <v>45.1</v>
+        <v>42.7</v>
       </c>
     </row>
   </sheetData>
@@ -1151,25 +1151,25 @@
         <v>11</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L2">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M2">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="N2">
-        <v>131</v>
+        <v>158</v>
       </c>
       <c r="O2">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="P2" s="1">
-        <v>44.3</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -1257,19 +1257,19 @@
         <v>2</v>
       </c>
       <c r="L4">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>187</v>
+        <v>26</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>174</v>
       </c>
       <c r="O4">
-        <v>210</v>
+        <v>36</v>
       </c>
       <c r="P4" s="1">
-        <v>100</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -1301,25 +1301,25 @@
         <v>13</v>
       </c>
       <c r="J5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L5">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M5">
-        <v>253</v>
+        <v>69</v>
       </c>
       <c r="N5">
-        <v>279</v>
+        <v>480</v>
       </c>
       <c r="O5">
-        <v>350</v>
+        <v>149</v>
       </c>
       <c r="P5" s="1">
-        <v>55.6</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1339,37 +1339,37 @@
         <v>0</v>
       </c>
       <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
         <v>6</v>
       </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
       <c r="H6">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="I6">
         <v>15</v>
       </c>
       <c r="J6">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L6">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="M6">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N6">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="O6">
-        <v>130</v>
+        <v>97</v>
       </c>
       <c r="P6" s="1">
-        <v>87.2</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -1489,37 +1489,37 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H9">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="I9">
         <v>17</v>
       </c>
       <c r="J9">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="K9">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L9">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="M9">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N9">
-        <v>160</v>
+        <v>193</v>
       </c>
       <c r="O9">
-        <v>201</v>
+        <v>168</v>
       </c>
       <c r="P9" s="1">
-        <v>55.7</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -1536,37 +1536,37 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H10">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="I10">
         <v>30</v>
       </c>
       <c r="J10">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="K10">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L10">
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="M10">
-        <v>308</v>
+        <v>125</v>
       </c>
       <c r="N10">
-        <v>439</v>
+        <v>673</v>
       </c>
       <c r="O10">
-        <v>551</v>
+        <v>317</v>
       </c>
       <c r="P10" s="1">
-        <v>55.7</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1661,25 +1661,25 @@
         <v>10</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L2">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="M2">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="N2">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="O2">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="P2" s="1">
-        <v>46</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -1767,19 +1767,19 @@
         <v>2</v>
       </c>
       <c r="L4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="N4">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="O4">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="P4" s="1">
-        <v>27.1</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -1811,25 +1811,25 @@
         <v>14</v>
       </c>
       <c r="J5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K5">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="L5">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="M5">
-        <v>234</v>
+        <v>208</v>
       </c>
       <c r="N5">
-        <v>280</v>
+        <v>322</v>
       </c>
       <c r="O5">
-        <v>349</v>
+        <v>307</v>
       </c>
       <c r="P5" s="1">
-        <v>55.5</v>
+        <v>48.8</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1849,37 +1849,37 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J6">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K6">
         <v>17</v>
       </c>
       <c r="L6">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M6">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="N6">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="O6">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="P6" s="1">
-        <v>63.1</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -1999,37 +1999,37 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I9">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J9">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K9">
         <v>32</v>
       </c>
       <c r="L9">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M9">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="N9">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="O9">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="P9" s="1">
-        <v>61.8</v>
+        <v>62.6</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -2046,37 +2046,37 @@
         <v>0</v>
       </c>
       <c r="F10">
+        <v>11</v>
+      </c>
+      <c r="G10">
         <v>5</v>
       </c>
-      <c r="G10">
-        <v>8</v>
-      </c>
       <c r="H10">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="I10">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J10">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="K10">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L10">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="M10">
-        <v>326</v>
+        <v>301</v>
       </c>
       <c r="N10">
-        <v>418</v>
+        <v>457</v>
       </c>
       <c r="O10">
-        <v>572</v>
+        <v>533</v>
       </c>
       <c r="P10" s="1">
-        <v>57.8</v>
+        <v>53.8</v>
       </c>
     </row>
   </sheetData>
@@ -2212,25 +2212,25 @@
         <v>1</v>
       </c>
       <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
         <v>5</v>
       </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
       <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
         <v>9</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>21</v>
       </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
       <c r="N3">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="O3" s="1">
-        <v>100</v>
+        <v>48.8</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -2735,19 +2735,19 @@
         <v>0</v>
       </c>
       <c r="K14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L14">
         <v>3</v>
       </c>
       <c r="M14">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="N14">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O14" s="1">
-        <v>32.1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -2782,19 +2782,19 @@
         <v>0</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L15">
+        <v>4</v>
+      </c>
+      <c r="M15">
+        <v>36</v>
+      </c>
+      <c r="N15">
         <v>5</v>
       </c>
-      <c r="M15">
-        <v>34</v>
-      </c>
-      <c r="N15">
-        <v>7</v>
-      </c>
       <c r="O15" s="1">
-        <v>17.1</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -2829,19 +2829,19 @@
         <v>0</v>
       </c>
       <c r="K16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L16">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M16">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="N16">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="O16" s="1">
-        <v>35.3</v>
+        <v>26.5</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -2879,16 +2879,16 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="M17">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="N17">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="O17" s="1">
-        <v>32.5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -2923,19 +2923,19 @@
         <v>2</v>
       </c>
       <c r="K18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M18">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="N18">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="O18" s="1">
-        <v>35.5</v>
+        <v>22.6</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -2973,16 +2973,16 @@
         <v>0</v>
       </c>
       <c r="L19">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M19">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="N19">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O19" s="1">
-        <v>13.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -3005,19 +3005,19 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H20">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I20">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J20">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L20">
         <v>10</v>
@@ -3046,28 +3046,28 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F21">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21">
         <v>3</v>
       </c>
       <c r="I21">
+        <v>8</v>
+      </c>
+      <c r="J21">
         <v>6</v>
       </c>
-      <c r="J21">
-        <v>7</v>
-      </c>
       <c r="K21">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M21">
         <v>7</v>
@@ -3093,37 +3093,37 @@
         <v>0</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F22">
         <v>1</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H22">
         <v>1</v>
       </c>
       <c r="I22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J22">
         <v>1</v>
       </c>
       <c r="K22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M22">
+        <v>15</v>
+      </c>
+      <c r="N22">
         <v>18</v>
       </c>
-      <c r="N22">
-        <v>15</v>
-      </c>
       <c r="O22" s="1">
-        <v>45.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -3763,22 +3763,22 @@
         <v>41</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F3" s="1">
-        <v>0</v>
+        <v>56.1</v>
       </c>
       <c r="G3" s="1">
-        <v>0</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="H3" s="1">
-        <v>0</v>
+        <v>51.2</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -4052,19 +4052,19 @@
         <v>19</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E14">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F14" s="1">
         <v>67.90000000000001</v>
       </c>
       <c r="G14" s="1">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H14" s="1">
-        <v>67.90000000000001</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -4078,19 +4078,19 @@
         <v>33</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E15">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F15" s="1">
         <v>80.5</v>
       </c>
       <c r="G15" s="1">
-        <v>0</v>
+        <v>87.8</v>
       </c>
       <c r="H15" s="1">
-        <v>82.90000000000001</v>
+        <v>87.8</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -4104,19 +4104,19 @@
         <v>20</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E16">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F16" s="1">
         <v>58.8</v>
       </c>
       <c r="G16" s="1">
-        <v>0</v>
+        <v>73.5</v>
       </c>
       <c r="H16" s="1">
-        <v>64.7</v>
+        <v>73.5</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -4130,19 +4130,19 @@
         <v>27</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E17">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F17" s="1">
         <v>67.5</v>
       </c>
       <c r="G17" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H17" s="1">
-        <v>67.5</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -4156,19 +4156,19 @@
         <v>18</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E18">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F18" s="1">
         <v>58.1</v>
       </c>
       <c r="G18" s="1">
-        <v>0</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="H18" s="1">
-        <v>64.5</v>
+        <v>77.40000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -4182,19 +4182,19 @@
         <v>31</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E19">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F19" s="1">
         <v>86.09999999999999</v>
       </c>
       <c r="G19" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H19" s="1">
-        <v>86.09999999999999</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -4208,7 +4208,7 @@
         <v>4</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E20">
         <v>11</v>
@@ -4217,7 +4217,7 @@
         <v>10</v>
       </c>
       <c r="G20" s="1">
-        <v>0</v>
+        <v>27.5</v>
       </c>
       <c r="H20" s="1">
         <v>27.5</v>
@@ -4234,7 +4234,7 @@
         <v>7</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E21">
         <v>7</v>
@@ -4243,7 +4243,7 @@
         <v>20.6</v>
       </c>
       <c r="G21" s="1">
-        <v>0</v>
+        <v>20.6</v>
       </c>
       <c r="H21" s="1">
         <v>20.6</v>
@@ -4260,19 +4260,19 @@
         <v>12</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E22">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F22" s="1">
         <v>36.4</v>
       </c>
       <c r="G22" s="1">
-        <v>0</v>
+        <v>45.5</v>
       </c>
       <c r="H22" s="1">
-        <v>54.5</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="23" spans="1:8">

</xml_diff>

<commit_message>
Estadisticos Segundo Parcial 20241 Sin RS
</commit_message>
<xml_diff>
--- a/Totales Generales20241.xlsx
+++ b/Totales Generales20241.xlsx
@@ -650,16 +650,16 @@
         <v>23</v>
       </c>
       <c r="M2">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="P2" s="1">
-        <v>36.6</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -685,19 +685,19 @@
         <v>0</v>
       </c>
       <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
         <v>3</v>
       </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
       <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L3">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M3">
         <v>24</v>
@@ -785,31 +785,31 @@
         <v>4</v>
       </c>
       <c r="H5">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J5">
         <v>14</v>
       </c>
       <c r="K5">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L5">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="M5">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N5">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="O5">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P5" s="1">
-        <v>32.8</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1032,31 +1032,31 @@
         <v>14</v>
       </c>
       <c r="H10">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I10">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J10">
         <v>37</v>
       </c>
       <c r="K10">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L10">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M10">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="N10">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="O10">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="P10" s="1">
-        <v>42.7</v>
+        <v>42.6</v>
       </c>
     </row>
   </sheetData>
@@ -1649,37 +1649,37 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L2">
         <v>18</v>
       </c>
       <c r="M2">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="N2">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="O2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="P2" s="1">
-        <v>37</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -1699,37 +1699,37 @@
         <v>0</v>
       </c>
       <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
         <v>1</v>
       </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
         <v>13</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>18</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>148</v>
       </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
       <c r="O3">
-        <v>184</v>
+        <v>36</v>
       </c>
       <c r="P3" s="1">
-        <v>100</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -1799,37 +1799,37 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K5">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="L5">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="M5">
-        <v>208</v>
+        <v>69</v>
       </c>
       <c r="N5">
-        <v>322</v>
+        <v>480</v>
       </c>
       <c r="O5">
-        <v>307</v>
+        <v>149</v>
       </c>
       <c r="P5" s="1">
-        <v>48.8</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1849,16 +1849,16 @@
         <v>0</v>
       </c>
       <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
         <v>6</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
       <c r="H6">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I6">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J6">
         <v>17</v>
@@ -1867,10 +1867,10 @@
         <v>17</v>
       </c>
       <c r="L6">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M6">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="N6">
         <v>52</v>
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7">
         <v>2</v>
@@ -1908,28 +1908,28 @@
         <v>2</v>
       </c>
       <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
         <v>5</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>1</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>7</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>19</v>
       </c>
-      <c r="M7">
-        <v>58</v>
-      </c>
       <c r="N7">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="O7">
-        <v>96</v>
+        <v>38</v>
       </c>
       <c r="P7" s="1">
-        <v>99</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -1999,37 +1999,37 @@
         <v>0</v>
       </c>
       <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
         <v>8</v>
       </c>
-      <c r="G9">
-        <v>3</v>
-      </c>
       <c r="H9">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I9">
         <v>17</v>
       </c>
       <c r="J9">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K9">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="L9">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="M9">
-        <v>93</v>
+        <v>56</v>
       </c>
       <c r="N9">
-        <v>135</v>
+        <v>193</v>
       </c>
       <c r="O9">
-        <v>226</v>
+        <v>168</v>
       </c>
       <c r="P9" s="1">
-        <v>62.6</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -2046,37 +2046,37 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="H10">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="I10">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J10">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="K10">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="L10">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="M10">
-        <v>301</v>
+        <v>125</v>
       </c>
       <c r="N10">
-        <v>457</v>
+        <v>673</v>
       </c>
       <c r="O10">
-        <v>533</v>
+        <v>317</v>
       </c>
       <c r="P10" s="1">
-        <v>53.8</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -2159,13 +2159,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H2">
         <v>3</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -2174,16 +2174,16 @@
         <v>2</v>
       </c>
       <c r="L2">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M2">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="N2">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="O2" s="1">
-        <v>47.5</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -2200,10 +2200,10 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2215,22 +2215,22 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K3">
         <v>2</v>
       </c>
       <c r="L3">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="M3">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="N3">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="O3" s="1">
-        <v>48.8</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -2253,10 +2253,10 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -2444,7 +2444,7 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -2453,19 +2453,19 @@
         <v>1</v>
       </c>
       <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8">
         <v>5</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>16</v>
       </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
       <c r="N8">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="O8" s="1">
-        <v>100</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -2497,22 +2497,22 @@
         <v>0</v>
       </c>
       <c r="J9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K9">
         <v>4</v>
       </c>
       <c r="L9">
+        <v>4</v>
+      </c>
+      <c r="M9">
         <v>28</v>
       </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
       <c r="N9">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="O9" s="1">
-        <v>100</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -2529,11 +2529,11 @@
         <v>0</v>
       </c>
       <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
         <v>1</v>
       </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
       <c r="G10">
         <v>0</v>
       </c>
@@ -2541,25 +2541,25 @@
         <v>0</v>
       </c>
       <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
         <v>1</v>
       </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
         <v>26</v>
       </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
       <c r="N10">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="O10" s="1">
-        <v>100</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -2585,28 +2585,28 @@
         <v>0</v>
       </c>
       <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
         <v>1</v>
       </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
       <c r="J11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K11">
+        <v>2</v>
+      </c>
+      <c r="L11">
         <v>3</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>29</v>
       </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
       <c r="N11">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="O11" s="1">
-        <v>100</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -2638,22 +2638,22 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K12">
         <v>4</v>
       </c>
       <c r="L12">
+        <v>4</v>
+      </c>
+      <c r="M12">
         <v>16</v>
       </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
       <c r="N12">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="O12" s="1">
-        <v>100</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -2685,22 +2685,22 @@
         <v>0</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K13">
         <v>2</v>
       </c>
       <c r="L13">
+        <v>2</v>
+      </c>
+      <c r="M13">
         <v>33</v>
       </c>
-      <c r="M13">
-        <v>0</v>
-      </c>
       <c r="N13">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="O13" s="1">
-        <v>100</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -3005,19 +3005,19 @@
         <v>0</v>
       </c>
       <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>6</v>
+      </c>
+      <c r="I20">
         <v>4</v>
       </c>
-      <c r="H20">
-        <v>4</v>
-      </c>
-      <c r="I20">
-        <v>3</v>
-      </c>
       <c r="J20">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L20">
         <v>10</v>
@@ -3046,28 +3046,28 @@
         <v>0</v>
       </c>
       <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
         <v>3</v>
       </c>
-      <c r="F21">
-        <v>0</v>
-      </c>
       <c r="G21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21">
         <v>3</v>
       </c>
       <c r="I21">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J21">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K21">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21">
         <v>7</v>
@@ -3093,28 +3093,28 @@
         <v>0</v>
       </c>
       <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
         <v>3</v>
       </c>
-      <c r="F22">
+      <c r="G22">
         <v>1</v>
       </c>
-      <c r="G22">
-        <v>2</v>
-      </c>
       <c r="H22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J22">
         <v>1</v>
       </c>
       <c r="K22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M22">
         <v>15</v>
@@ -3234,37 +3234,37 @@
         <v>0</v>
       </c>
       <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
         <v>1</v>
       </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
       <c r="G25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H25">
+        <v>2</v>
+      </c>
+      <c r="I25">
         <v>4</v>
       </c>
-      <c r="I25">
-        <v>0</v>
-      </c>
       <c r="J25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K25">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L25">
         <v>6</v>
       </c>
       <c r="M25">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N25">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="O25" s="1">
-        <v>95.5</v>
+        <v>68.2</v>
       </c>
     </row>
     <row r="26" spans="1:15">
@@ -3284,34 +3284,34 @@
         <v>0</v>
       </c>
       <c r="F26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H26">
         <v>0</v>
       </c>
       <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
         <v>1</v>
       </c>
-      <c r="J26">
-        <v>2</v>
-      </c>
       <c r="K26">
+        <v>2</v>
+      </c>
+      <c r="L26">
         <v>4</v>
       </c>
-      <c r="L26">
+      <c r="M26">
         <v>16</v>
       </c>
-      <c r="M26">
-        <v>0</v>
-      </c>
       <c r="N26">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="O26" s="1">
-        <v>100</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -3328,37 +3328,37 @@
         <v>0</v>
       </c>
       <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
         <v>1</v>
       </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
       <c r="G27">
         <v>0</v>
       </c>
       <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
         <v>1</v>
       </c>
-      <c r="I27">
-        <v>0</v>
-      </c>
       <c r="J27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K27">
+        <v>2</v>
+      </c>
+      <c r="L27">
         <v>4</v>
       </c>
-      <c r="L27">
+      <c r="M27">
         <v>11</v>
       </c>
-      <c r="M27">
-        <v>0</v>
-      </c>
       <c r="N27">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="O27" s="1">
-        <v>100</v>
+        <v>42.1</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -3390,22 +3390,22 @@
         <v>0</v>
       </c>
       <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
         <v>1</v>
       </c>
-      <c r="K28">
+      <c r="L28">
         <v>3</v>
       </c>
-      <c r="L28">
+      <c r="M28">
         <v>17</v>
       </c>
-      <c r="M28">
-        <v>0</v>
-      </c>
       <c r="N28">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="O28" s="1">
-        <v>100</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:15">
@@ -3440,19 +3440,19 @@
         <v>0</v>
       </c>
       <c r="K29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L29">
+        <v>2</v>
+      </c>
+      <c r="M29">
         <v>8</v>
       </c>
-      <c r="M29">
-        <v>0</v>
-      </c>
       <c r="N29">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O29" s="1">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:15">
@@ -3737,22 +3737,22 @@
         <v>40</v>
       </c>
       <c r="C2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D2">
         <v>25</v>
       </c>
       <c r="E2">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F2" s="1">
-        <v>60</v>
+        <v>62.5</v>
       </c>
       <c r="G2" s="1">
         <v>62.5</v>
       </c>
       <c r="H2" s="1">
-        <v>52.5</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -3769,7 +3769,7 @@
         <v>27</v>
       </c>
       <c r="E3">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F3" s="1">
         <v>56.1</v>
@@ -3778,7 +3778,7 @@
         <v>65.90000000000001</v>
       </c>
       <c r="H3" s="1">
-        <v>51.2</v>
+        <v>65.90000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -3899,7 +3899,7 @@
         <v>16</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F8" s="1">
         <v>41.7</v>
@@ -3908,7 +3908,7 @@
         <v>66.7</v>
       </c>
       <c r="H8" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3925,7 +3925,7 @@
         <v>28</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F9" s="1">
         <v>50</v>
@@ -3934,7 +3934,7 @@
         <v>77.8</v>
       </c>
       <c r="H9" s="1">
-        <v>0</v>
+        <v>77.8</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -3951,7 +3951,7 @@
         <v>26</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F10" s="1">
         <v>89.3</v>
@@ -3960,7 +3960,7 @@
         <v>92.90000000000001</v>
       </c>
       <c r="H10" s="1">
-        <v>0</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -3977,7 +3977,7 @@
         <v>29</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F11" s="1">
         <v>80</v>
@@ -3986,7 +3986,7 @@
         <v>82.90000000000001</v>
       </c>
       <c r="H11" s="1">
-        <v>0</v>
+        <v>82.90000000000001</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -4003,7 +4003,7 @@
         <v>16</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F12" s="1">
         <v>62.5</v>
@@ -4012,7 +4012,7 @@
         <v>66.7</v>
       </c>
       <c r="H12" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -4029,7 +4029,7 @@
         <v>33</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F13" s="1">
         <v>81.09999999999999</v>
@@ -4038,7 +4038,7 @@
         <v>89.2</v>
       </c>
       <c r="H13" s="1">
-        <v>0</v>
+        <v>89.2</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -4341,7 +4341,7 @@
         <v>7</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F25" s="1">
         <v>27.3</v>
@@ -4350,7 +4350,7 @@
         <v>31.8</v>
       </c>
       <c r="H25" s="1">
-        <v>4.5</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -4367,7 +4367,7 @@
         <v>16</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F26" s="1">
         <v>28</v>
@@ -4376,7 +4376,7 @@
         <v>64</v>
       </c>
       <c r="H26" s="1">
-        <v>0</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -4393,7 +4393,7 @@
         <v>11</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F27" s="1">
         <v>52.6</v>
@@ -4402,7 +4402,7 @@
         <v>57.9</v>
       </c>
       <c r="H27" s="1">
-        <v>0</v>
+        <v>57.9</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -4419,7 +4419,7 @@
         <v>17</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F28" s="1">
         <v>71.40000000000001</v>
@@ -4428,7 +4428,7 @@
         <v>81</v>
       </c>
       <c r="H28" s="1">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -4445,7 +4445,7 @@
         <v>8</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F29" s="1">
         <v>50</v>
@@ -4454,7 +4454,7 @@
         <v>80</v>
       </c>
       <c r="H29" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="30" spans="1:8">

</xml_diff>

<commit_message>
Estadisticos Tercer Parcial 9Dic
</commit_message>
<xml_diff>
--- a/Totales Generales20241.xlsx
+++ b/Totales Generales20241.xlsx
@@ -720,7 +720,7 @@
         <v>17</v>
       </c>
       <c r="C4">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -735,7 +735,7 @@
         <v>1</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I4">
         <v>3</v>
@@ -744,7 +744,7 @@
         <v>4</v>
       </c>
       <c r="K4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L4">
         <v>11</v>
@@ -756,10 +756,10 @@
         <v>148</v>
       </c>
       <c r="O4">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="P4" s="1">
-        <v>29.5</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -770,7 +770,7 @@
         <v>17</v>
       </c>
       <c r="C5">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -785,7 +785,7 @@
         <v>4</v>
       </c>
       <c r="H5">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I5">
         <v>14</v>
@@ -794,7 +794,7 @@
         <v>14</v>
       </c>
       <c r="K5">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="L5">
         <v>56</v>
@@ -806,10 +806,10 @@
         <v>424</v>
       </c>
       <c r="O5">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="P5" s="1">
-        <v>32.6</v>
+        <v>33.1</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -850,16 +850,16 @@
         <v>21</v>
       </c>
       <c r="M6">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="N6">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="O6">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="P6" s="1">
-        <v>74.5</v>
+        <v>73.2</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -920,7 +920,7 @@
         <v>18</v>
       </c>
       <c r="C8">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -935,13 +935,13 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K8">
         <v>15</v>
@@ -956,10 +956,10 @@
         <v>63</v>
       </c>
       <c r="O8">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="P8" s="1">
-        <v>45.2</v>
+        <v>47.9</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -970,7 +970,7 @@
         <v>18</v>
       </c>
       <c r="C9">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -985,13 +985,13 @@
         <v>10</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I9">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J9">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="K9">
         <v>37</v>
@@ -1000,16 +1000,16 @@
         <v>45</v>
       </c>
       <c r="M9">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="N9">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="O9">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="P9" s="1">
-        <v>60.1</v>
+        <v>60.2</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -1017,7 +1017,7 @@
         <v>16</v>
       </c>
       <c r="C10">
-        <v>990</v>
+        <v>1001</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -1032,31 +1032,31 @@
         <v>14</v>
       </c>
       <c r="H10">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I10">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J10">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="K10">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L10">
         <v>101</v>
       </c>
       <c r="M10">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="N10">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="O10">
-        <v>422</v>
+        <v>431</v>
       </c>
       <c r="P10" s="1">
-        <v>42.6</v>
+        <v>43.1</v>
       </c>
     </row>
   </sheetData>
@@ -1154,22 +1154,22 @@
         <v>4</v>
       </c>
       <c r="K2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O2">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="P2" s="1">
-        <v>32.8</v>
+        <v>32.3</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -1230,7 +1230,7 @@
         <v>17</v>
       </c>
       <c r="C4">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -1245,7 +1245,7 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4">
         <v>2</v>
@@ -1254,22 +1254,22 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N4">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="O4">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="P4" s="1">
-        <v>17.1</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -1280,7 +1280,7 @@
         <v>17</v>
       </c>
       <c r="C5">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1295,7 +1295,7 @@
         <v>5</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I5">
         <v>13</v>
@@ -1304,22 +1304,22 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="L5">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M5">
         <v>69</v>
       </c>
       <c r="N5">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="O5">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="P5" s="1">
-        <v>23.7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1430,7 +1430,7 @@
         <v>18</v>
       </c>
       <c r="C8">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -1445,13 +1445,13 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K8">
         <v>8</v>
@@ -1466,10 +1466,10 @@
         <v>82</v>
       </c>
       <c r="O8">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="P8" s="1">
-        <v>28.7</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -1480,7 +1480,7 @@
         <v>18</v>
       </c>
       <c r="C9">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -1495,13 +1495,13 @@
         <v>8</v>
       </c>
       <c r="H9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J9">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="K9">
         <v>26</v>
@@ -1516,10 +1516,10 @@
         <v>193</v>
       </c>
       <c r="O9">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="P9" s="1">
-        <v>46.5</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -1527,7 +1527,7 @@
         <v>16</v>
       </c>
       <c r="C10">
-        <v>990</v>
+        <v>1001</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -1542,31 +1542,31 @@
         <v>13</v>
       </c>
       <c r="H10">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I10">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J10">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="K10">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L10">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M10">
         <v>125</v>
       </c>
       <c r="N10">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="O10">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="P10" s="1">
-        <v>32</v>
+        <v>32.6</v>
       </c>
     </row>
   </sheetData>
@@ -1652,34 +1652,34 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H2">
         <v>4</v>
       </c>
       <c r="I2">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K2">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="L2">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M2">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="N2">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="O2">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="P2" s="1">
-        <v>32.8</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -1711,25 +1711,25 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="M3">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N3">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="O3">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="P3" s="1">
-        <v>19.6</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -1740,7 +1740,7 @@
         <v>17</v>
       </c>
       <c r="C4">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -1761,25 +1761,25 @@
         <v>2</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M4">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="N4">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="O4">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="P4" s="1">
-        <v>17.1</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -1790,7 +1790,7 @@
         <v>17</v>
       </c>
       <c r="C5">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1802,16 +1802,16 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H5">
         <v>5</v>
       </c>
       <c r="I5">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="J5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K5">
         <v>15</v>
@@ -1820,16 +1820,16 @@
         <v>36</v>
       </c>
       <c r="M5">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N5">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="O5">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="P5" s="1">
-        <v>23.7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1852,34 +1852,34 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
         <v>4</v>
       </c>
-      <c r="I6">
-        <v>15</v>
-      </c>
-      <c r="J6">
-        <v>17</v>
-      </c>
       <c r="K6">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="L6">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="M6">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="N6">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="O6">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="P6" s="1">
-        <v>65.09999999999999</v>
+        <v>58.4</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -1911,25 +1911,25 @@
         <v>2</v>
       </c>
       <c r="J7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M7">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="N7">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="O7">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="P7" s="1">
-        <v>39.2</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -1940,7 +1940,7 @@
         <v>18</v>
       </c>
       <c r="C8">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -1958,28 +1958,28 @@
         <v>2</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
+        <v>5</v>
+      </c>
+      <c r="K8">
         <v>4</v>
       </c>
-      <c r="K8">
-        <v>8</v>
-      </c>
       <c r="L8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N8">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="O8">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="P8" s="1">
-        <v>28.7</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -1990,7 +1990,7 @@
         <v>18</v>
       </c>
       <c r="C9">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -2002,34 +2002,34 @@
         <v>0</v>
       </c>
       <c r="G9">
+        <v>7</v>
+      </c>
+      <c r="H9">
+        <v>5</v>
+      </c>
+      <c r="I9">
         <v>8</v>
       </c>
-      <c r="H9">
-        <v>8</v>
-      </c>
-      <c r="I9">
-        <v>17</v>
-      </c>
       <c r="J9">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="K9">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="L9">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="M9">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N9">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="O9">
-        <v>168</v>
+        <v>145</v>
       </c>
       <c r="P9" s="1">
-        <v>46.5</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -2037,7 +2037,7 @@
         <v>16</v>
       </c>
       <c r="C10">
-        <v>990</v>
+        <v>1001</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -2049,34 +2049,34 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H10">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I10">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="J10">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="K10">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="L10">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="M10">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="N10">
-        <v>673</v>
+        <v>710</v>
       </c>
       <c r="O10">
-        <v>317</v>
+        <v>291</v>
       </c>
       <c r="P10" s="1">
-        <v>32</v>
+        <v>29.1</v>
       </c>
     </row>
   </sheetData>
@@ -2159,31 +2159,31 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
         <v>3</v>
       </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L2">
         <v>6</v>
       </c>
       <c r="M2">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="N2">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O2" s="1">
-        <v>37.5</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -2209,19 +2209,19 @@
         <v>0</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M3">
         <v>27</v>
@@ -2256,16 +2256,16 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4">
         <v>8</v>
@@ -2300,13 +2300,13 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -2344,34 +2344,34 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6">
         <v>3</v>
       </c>
       <c r="L6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N6">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O6" s="1">
-        <v>35.1</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -2394,22 +2394,22 @@
         <v>0</v>
       </c>
       <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
         <v>2</v>
       </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>1</v>
-      </c>
-      <c r="K7">
+      <c r="L7">
         <v>3</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
       </c>
       <c r="M7">
         <v>25</v>
@@ -2447,25 +2447,25 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <v>1</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M8">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O8" s="1">
-        <v>33.3</v>
+        <v>29.2</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -2497,13 +2497,13 @@
         <v>0</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M9">
         <v>28</v>
@@ -2544,10 +2544,10 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -2588,25 +2588,25 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
         <v>2</v>
       </c>
-      <c r="L11">
-        <v>3</v>
-      </c>
       <c r="M11">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="N11">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O11" s="1">
-        <v>17.1</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -2641,10 +2641,10 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M12">
         <v>16</v>
@@ -2691,16 +2691,16 @@
         <v>2</v>
       </c>
       <c r="L13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M13">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O13" s="1">
-        <v>10.8</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -2708,7 +2708,7 @@
         <v>32</v>
       </c>
       <c r="B14">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -2723,7 +2723,7 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -2744,10 +2744,10 @@
         <v>21</v>
       </c>
       <c r="N14">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O14" s="1">
-        <v>25</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -2817,31 +2817,31 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16">
         <v>1</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16">
         <v>0</v>
       </c>
       <c r="K16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16">
         <v>6</v>
       </c>
       <c r="M16">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N16">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O16" s="1">
-        <v>26.5</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -2849,7 +2849,7 @@
         <v>35</v>
       </c>
       <c r="B17">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -2873,22 +2873,22 @@
         <v>0</v>
       </c>
       <c r="J17">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L17">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M17">
         <v>32</v>
       </c>
       <c r="N17">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="O17" s="1">
-        <v>20</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -3005,31 +3005,31 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J20">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K20">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L20">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M20">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="N20">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="O20" s="1">
-        <v>72.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -3049,34 +3049,34 @@
         <v>0</v>
       </c>
       <c r="F21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G21">
         <v>0</v>
       </c>
       <c r="H21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
         <v>6</v>
       </c>
-      <c r="J21">
+      <c r="K21">
+        <v>8</v>
+      </c>
+      <c r="L21">
         <v>7</v>
       </c>
-      <c r="K21">
-        <v>7</v>
-      </c>
-      <c r="L21">
-        <v>1</v>
-      </c>
       <c r="M21">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N21">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="O21" s="1">
-        <v>79.40000000000001</v>
+        <v>73.5</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -3102,28 +3102,28 @@
         <v>1</v>
       </c>
       <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
         <v>2</v>
       </c>
-      <c r="I22">
-        <v>2</v>
-      </c>
-      <c r="J22">
-        <v>1</v>
-      </c>
       <c r="K22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L22">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M22">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N22">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="O22" s="1">
-        <v>54.5</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -3146,31 +3146,31 @@
         <v>0</v>
       </c>
       <c r="G23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K23">
         <v>3</v>
       </c>
       <c r="L23">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M23">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="N23">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="O23" s="1">
-        <v>73.90000000000001</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -3196,19 +3196,19 @@
         <v>0</v>
       </c>
       <c r="H24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
         <v>2</v>
       </c>
-      <c r="J24">
-        <v>0</v>
-      </c>
-      <c r="K24">
-        <v>0</v>
-      </c>
       <c r="L24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M24">
         <v>13</v>
@@ -3299,19 +3299,19 @@
         <v>1</v>
       </c>
       <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
         <v>2</v>
       </c>
-      <c r="L26">
-        <v>4</v>
-      </c>
       <c r="M26">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="N26">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="O26" s="1">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -3340,25 +3340,25 @@
         <v>0</v>
       </c>
       <c r="I27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27">
         <v>0</v>
       </c>
       <c r="K27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L27">
+        <v>3</v>
+      </c>
+      <c r="M27">
+        <v>15</v>
+      </c>
+      <c r="N27">
         <v>4</v>
       </c>
-      <c r="M27">
-        <v>11</v>
-      </c>
-      <c r="N27">
-        <v>8</v>
-      </c>
       <c r="O27" s="1">
-        <v>42.1</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -3390,22 +3390,22 @@
         <v>0</v>
       </c>
       <c r="J28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28">
         <v>1</v>
       </c>
       <c r="L28">
+        <v>1</v>
+      </c>
+      <c r="M28">
+        <v>18</v>
+      </c>
+      <c r="N28">
         <v>3</v>
       </c>
-      <c r="M28">
-        <v>17</v>
-      </c>
-      <c r="N28">
-        <v>4</v>
-      </c>
       <c r="O28" s="1">
-        <v>19</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="29" spans="1:15">
@@ -3443,16 +3443,16 @@
         <v>0</v>
       </c>
       <c r="L29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M29">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O29" s="1">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:15">
@@ -3460,7 +3460,7 @@
         <v>48</v>
       </c>
       <c r="B30">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -3484,22 +3484,22 @@
         <v>0</v>
       </c>
       <c r="J30">
+        <v>1</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="L30">
         <v>5</v>
       </c>
-      <c r="K30">
-        <v>2</v>
-      </c>
-      <c r="L30">
-        <v>3</v>
-      </c>
       <c r="M30">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="N30">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="O30" s="1">
-        <v>52.4</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="31" spans="1:15">
@@ -3528,13 +3528,13 @@
         <v>0</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31">
+        <v>3</v>
+      </c>
+      <c r="K31">
         <v>2</v>
-      </c>
-      <c r="K31">
-        <v>4</v>
       </c>
       <c r="L31">
         <v>3</v>
@@ -3575,16 +3575,16 @@
         <v>0</v>
       </c>
       <c r="I32">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L32">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M32">
         <v>13</v>
@@ -3601,7 +3601,7 @@
         <v>51</v>
       </c>
       <c r="B33">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -3619,7 +3619,7 @@
         <v>0</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33">
         <v>0</v>
@@ -3628,19 +3628,19 @@
         <v>0</v>
       </c>
       <c r="K33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L33">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M33">
         <v>19</v>
       </c>
       <c r="N33">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O33" s="1">
-        <v>17.4</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="34" spans="1:15">
@@ -3648,46 +3648,46 @@
         <v>52</v>
       </c>
       <c r="B34">
+        <v>29</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <v>4</v>
+      </c>
+      <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="M34">
         <v>25</v>
       </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
-      <c r="D34">
-        <v>0</v>
-      </c>
-      <c r="E34">
-        <v>0</v>
-      </c>
-      <c r="F34">
-        <v>0</v>
-      </c>
-      <c r="G34">
-        <v>0</v>
-      </c>
-      <c r="H34">
-        <v>0</v>
-      </c>
-      <c r="I34">
-        <v>0</v>
-      </c>
-      <c r="J34">
-        <v>0</v>
-      </c>
-      <c r="K34">
-        <v>0</v>
-      </c>
-      <c r="L34">
-        <v>3</v>
-      </c>
-      <c r="M34">
-        <v>22</v>
-      </c>
       <c r="N34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O34" s="1">
-        <v>12</v>
+        <v>13.8</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="E2">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F2" s="1">
         <v>62.5</v>
@@ -3752,7 +3752,7 @@
         <v>62.5</v>
       </c>
       <c r="H2" s="1">
-        <v>62.5</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -3844,19 +3844,19 @@
         <v>24</v>
       </c>
       <c r="D6">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F6" s="1">
         <v>64.90000000000001</v>
       </c>
       <c r="G6" s="1">
-        <v>64.90000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="H6" s="1">
-        <v>64.90000000000001</v>
+        <v>67.59999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -3899,7 +3899,7 @@
         <v>16</v>
       </c>
       <c r="E8">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F8" s="1">
         <v>41.7</v>
@@ -3908,7 +3908,7 @@
         <v>66.7</v>
       </c>
       <c r="H8" s="1">
-        <v>66.7</v>
+        <v>70.8</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3977,7 +3977,7 @@
         <v>29</v>
       </c>
       <c r="E11">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F11" s="1">
         <v>80</v>
@@ -3986,7 +3986,7 @@
         <v>82.90000000000001</v>
       </c>
       <c r="H11" s="1">
-        <v>82.90000000000001</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -4029,7 +4029,7 @@
         <v>33</v>
       </c>
       <c r="E13">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F13" s="1">
         <v>81.09999999999999</v>
@@ -4038,7 +4038,7 @@
         <v>89.2</v>
       </c>
       <c r="H13" s="1">
-        <v>89.2</v>
+        <v>91.90000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -4046,7 +4046,7 @@
         <v>32</v>
       </c>
       <c r="B14">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14">
         <v>19</v>
@@ -4058,13 +4058,13 @@
         <v>21</v>
       </c>
       <c r="F14" s="1">
-        <v>67.90000000000001</v>
+        <v>65.5</v>
       </c>
       <c r="G14" s="1">
-        <v>75</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="H14" s="1">
-        <v>75</v>
+        <v>72.40000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -4104,19 +4104,19 @@
         <v>20</v>
       </c>
       <c r="D16">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E16">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F16" s="1">
         <v>58.8</v>
       </c>
       <c r="G16" s="1">
-        <v>73.5</v>
+        <v>76.5</v>
       </c>
       <c r="H16" s="1">
-        <v>73.5</v>
+        <v>76.5</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -4124,7 +4124,7 @@
         <v>35</v>
       </c>
       <c r="B17">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C17">
         <v>27</v>
@@ -4136,13 +4136,13 @@
         <v>32</v>
       </c>
       <c r="F17" s="1">
-        <v>67.5</v>
+        <v>61.4</v>
       </c>
       <c r="G17" s="1">
-        <v>80</v>
+        <v>72.7</v>
       </c>
       <c r="H17" s="1">
-        <v>80</v>
+        <v>72.7</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -4205,22 +4205,22 @@
         <v>40</v>
       </c>
       <c r="C20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D20">
         <v>11</v>
       </c>
       <c r="E20">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F20" s="1">
-        <v>10</v>
+        <v>12.5</v>
       </c>
       <c r="G20" s="1">
         <v>27.5</v>
       </c>
       <c r="H20" s="1">
-        <v>27.5</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -4237,7 +4237,7 @@
         <v>7</v>
       </c>
       <c r="E21">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F21" s="1">
         <v>20.6</v>
@@ -4246,7 +4246,7 @@
         <v>20.6</v>
       </c>
       <c r="H21" s="1">
-        <v>20.6</v>
+        <v>26.5</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -4257,22 +4257,22 @@
         <v>33</v>
       </c>
       <c r="C22">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D22">
         <v>15</v>
       </c>
       <c r="E22">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F22" s="1">
-        <v>36.4</v>
+        <v>39.4</v>
       </c>
       <c r="G22" s="1">
         <v>45.5</v>
       </c>
       <c r="H22" s="1">
-        <v>45.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -4289,7 +4289,7 @@
         <v>6</v>
       </c>
       <c r="E23">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F23" s="1">
         <v>21.7</v>
@@ -4298,7 +4298,7 @@
         <v>26.1</v>
       </c>
       <c r="H23" s="1">
-        <v>26.1</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -4367,7 +4367,7 @@
         <v>16</v>
       </c>
       <c r="E26">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F26" s="1">
         <v>28</v>
@@ -4376,7 +4376,7 @@
         <v>64</v>
       </c>
       <c r="H26" s="1">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -4393,7 +4393,7 @@
         <v>11</v>
       </c>
       <c r="E27">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F27" s="1">
         <v>52.6</v>
@@ -4402,7 +4402,7 @@
         <v>57.9</v>
       </c>
       <c r="H27" s="1">
-        <v>57.9</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -4419,7 +4419,7 @@
         <v>17</v>
       </c>
       <c r="E28">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F28" s="1">
         <v>71.40000000000001</v>
@@ -4428,7 +4428,7 @@
         <v>81</v>
       </c>
       <c r="H28" s="1">
-        <v>81</v>
+        <v>85.7</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -4445,7 +4445,7 @@
         <v>8</v>
       </c>
       <c r="E29">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F29" s="1">
         <v>50</v>
@@ -4454,7 +4454,7 @@
         <v>80</v>
       </c>
       <c r="H29" s="1">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -4462,7 +4462,7 @@
         <v>48</v>
       </c>
       <c r="B30">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C30">
         <v>8</v>
@@ -4471,16 +4471,16 @@
         <v>10</v>
       </c>
       <c r="E30">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F30" s="1">
-        <v>38.1</v>
+        <v>36.4</v>
       </c>
       <c r="G30" s="1">
-        <v>47.6</v>
+        <v>45.5</v>
       </c>
       <c r="H30" s="1">
-        <v>47.6</v>
+        <v>68.2</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -4540,7 +4540,7 @@
         <v>51</v>
       </c>
       <c r="B33">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C33">
         <v>17</v>
@@ -4552,13 +4552,13 @@
         <v>19</v>
       </c>
       <c r="F33" s="1">
-        <v>73.90000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="G33" s="1">
-        <v>82.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="H33" s="1">
-        <v>82.59999999999999</v>
+        <v>79.2</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -4566,7 +4566,7 @@
         <v>52</v>
       </c>
       <c r="B34">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C34">
         <v>15</v>
@@ -4575,16 +4575,16 @@
         <v>22</v>
       </c>
       <c r="E34">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F34" s="1">
-        <v>60</v>
+        <v>51.7</v>
       </c>
       <c r="G34" s="1">
-        <v>88</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="H34" s="1">
-        <v>88</v>
+        <v>86.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>